<commit_message>
Fix medium-severity audit findings
</commit_message>
<xml_diff>
--- a/planilhas_entrada/(MODELO) - TRANSFERENCIA SIMPRESS.xlsx
+++ b/planilhas_entrada/(MODELO) - TRANSFERENCIA SIMPRESS.xlsx
@@ -40,11 +40,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={60275236-4EFC-4994-9FDC-81FC2BC31C8B}</author>
-    <author>tc={6DADF1A5-C074-4ACF-AB6A-038F8D0E0DA4}</author>
-    <author>tc={F38182BE-F0DD-4FBF-BCBE-3CCD116706B4}</author>
-    <author>tc={27CDB7B3-072C-4787-A22C-924E48D622CB}</author>
-    <author>tc={5222E737-5F59-4E55-88B3-15225E40D31F}</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0" xr:uid="{60275236-4EFC-4994-9FDC-81FC2BC31C8B}">
@@ -96,11 +96,11 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={2CB11056-BD07-4F50-A42E-9CB81B4AB3F6}</author>
-    <author>tc={F6C1126D-2EAF-49C4-BC58-576BBAC5A91F}</author>
-    <author>tc={319494E5-ADDE-4536-B8D5-FB2F0CA05EEF}</author>
-    <author>tc={976F83BC-53BA-4FED-910E-F9F7870339E1}</author>
-    <author>tc={B80EE59B-AC0F-4C1D-A8BD-1F1036245D16}</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
+    <author>Instruções do formulário</author>
   </authors>
   <commentList>
     <comment ref="C4" authorId="0" shapeId="0" xr:uid="{2CB11056-BD07-4F50-A42E-9CB81B4AB3F6}">
@@ -741,7 +741,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Paula Caroline Evangelista" id="{E5D00606-8255-4657-8A77-F7CA63A5A882}" userId="S::pcevangelista@simpress.com.br::84545bca-1a0e-4693-a3d1-f4888da48560" providerId="AD"/>
+  <person displayName="Instruções do formulário" id="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" userId="simpress-template" providerId="None"/>
 </personList>
 </file>
 
@@ -1032,19 +1032,19 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B5" dT="2026-04-01T11:01:38.46" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{60275236-4EFC-4994-9FDC-81FC2BC31C8B}">
+  <threadedComment ref="B5" dT="2026-04-01T11:01:38.46" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{60275236-4EFC-4994-9FDC-81FC2BC31C8B}">
     <text>Nome do cliente</text>
   </threadedComment>
-  <threadedComment ref="J5" dT="2026-04-01T11:02:19.10" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{6DADF1A5-C074-4ACF-AB6A-038F8D0E0DA4}">
+  <threadedComment ref="J5" dT="2026-04-01T11:02:19.10" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{6DADF1A5-C074-4ACF-AB6A-038F8D0E0DA4}">
     <text>Número do contrato principal do cliente</text>
   </threadedComment>
-  <threadedComment ref="B7" dT="2026-04-01T11:03:21.70" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{F38182BE-F0DD-4FBF-BCBE-3CCD116706B4}">
+  <threadedComment ref="B7" dT="2026-04-01T11:03:21.70" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{F38182BE-F0DD-4FBF-BCBE-3CCD116706B4}">
     <text>Número de série na placa fixada no equipamento</text>
   </threadedComment>
-  <threadedComment ref="B15" dT="2026-04-01T11:04:15.78" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{27CDB7B3-072C-4787-A22C-924E48D622CB}">
+  <threadedComment ref="B15" dT="2026-04-01T11:04:15.78" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{27CDB7B3-072C-4787-A22C-924E48D622CB}">
     <text>Dados completos do local de instalação atual do equipamento</text>
   </threadedComment>
-  <threadedComment ref="B27" dT="2026-04-01T11:05:16.86" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{5222E737-5F59-4E55-88B3-15225E40D31F}">
+  <threadedComment ref="B27" dT="2026-04-01T11:05:16.86" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{5222E737-5F59-4E55-88B3-15225E40D31F}">
     <text xml:space="preserve">Dados completos do local de destino para a movimentação do equipamento.
 (CNPJ deve ser referente ao cadastro do endereço de destino)
 </text>
@@ -1054,23 +1054,23 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C4" dT="2026-04-01T11:06:06.76" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{2CB11056-BD07-4F50-A42E-9CB81B4AB3F6}">
+  <threadedComment ref="C4" dT="2026-04-01T11:06:06.76" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{2CB11056-BD07-4F50-A42E-9CB81B4AB3F6}">
     <text>Nome do cliente</text>
   </threadedComment>
-  <threadedComment ref="C5" dT="2026-04-01T11:06:19.75" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{F6C1126D-2EAF-49C4-BC58-576BBAC5A91F}">
+  <threadedComment ref="C5" dT="2026-04-01T11:06:19.75" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{F6C1126D-2EAF-49C4-BC58-576BBAC5A91F}">
     <text xml:space="preserve">Número do contrato principal do cliente
 </text>
   </threadedComment>
-  <threadedComment ref="C7" dT="2026-04-01T11:07:46.65" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{319494E5-ADDE-4536-B8D5-FB2F0CA05EEF}">
+  <threadedComment ref="C7" dT="2026-04-01T11:07:46.65" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{319494E5-ADDE-4536-B8D5-FB2F0CA05EEF}">
     <text xml:space="preserve">Dados completos do local de instalação atual do equipamento
 </text>
   </threadedComment>
-  <threadedComment ref="O7" dT="2026-04-01T11:08:03.53" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{976F83BC-53BA-4FED-910E-F9F7870339E1}">
+  <threadedComment ref="O7" dT="2026-04-01T11:08:03.53" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{976F83BC-53BA-4FED-910E-F9F7870339E1}">
     <text xml:space="preserve">Dados completos do local de destino para a movimentação do equipamento.
 (CNPJ deve ser referente ao cadastro do endereço de destino)
 </text>
   </threadedComment>
-  <threadedComment ref="B8" dT="2026-04-01T11:07:29.79" personId="{E5D00606-8255-4657-8A77-F7CA63A5A882}" id="{B80EE59B-AC0F-4C1D-A8BD-1F1036245D16}">
+  <threadedComment ref="B8" dT="2026-04-01T11:07:29.79" personId="{9176F3D8-D5D0-4CCD-8095-780E328A5694}" id="{B80EE59B-AC0F-4C1D-A8BD-1F1036245D16}">
     <text>Número de série na placa fixada no equipamento</text>
   </threadedComment>
 </ThreadedComments>

</xml_diff>

<commit_message>
Adiciona kit ao modelo de transferência
</commit_message>
<xml_diff>
--- a/planilhas_entrada/(MODELO) - TRANSFERENCIA SIMPRESS.xlsx
+++ b/planilhas_entrada/(MODELO) - TRANSFERENCIA SIMPRESS.xlsx
@@ -1208,7 +1208,11 @@
       <c r="C8" s="29"/>
       <c r="D8" s="29"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="26"/>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Notebook + kit na mochila</t>
+        </is>
+      </c>
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
       <c r="I8" s="3"/>

</xml_diff>